<commit_message>
Order of magnitude speedup using GPU and smarter CV calculations!
</commit_message>
<xml_diff>
--- a/history_matching/example/iter0/Cuts/RadiusShouldBe15/history_matching_config.xlsx
+++ b/history_matching/example/iter0/Cuts/RadiusShouldBe15/history_matching_config.xlsx
@@ -1,36 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="History_Matching_Params" sheetId="1" r:id="rId1"/>
-    <sheet name="Inputs" sheetId="2" r:id="rId2"/>
-    <sheet name="Results" sheetId="3" r:id="rId3"/>
-    <sheet name="Param_Info" sheetId="4" r:id="rId4"/>
+    <sheet name="History_Matching_Params" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Inputs" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Results" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Param_Info" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="47">
+  <si>
+    <t>Parameter</t>
+  </si>
   <si>
     <t>Value</t>
   </si>
   <si>
-    <t>Parameter</t>
-  </si>
-  <si>
     <t>cut_name</t>
   </si>
   <si>
+    <t>RadiusShouldBe15</t>
+  </si>
+  <si>
     <t>desired_result</t>
   </si>
   <si>
+    <t>desired_result_var</t>
+  </si>
+  <si>
     <t>discrepancy_var</t>
   </si>
   <si>
@@ -43,7 +49,7 @@
     <t>training_fraction</t>
   </si>
   <si>
-    <t>RadiusShouldBe15</t>
+    <t>Sample_Id</t>
   </si>
   <si>
     <t>Sample</t>
@@ -61,126 +67,119 @@
     <t>Train</t>
   </si>
   <si>
-    <t>Sample_Id</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000000</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000001</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000002</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000003</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000004</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000005</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000006</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000007</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000008</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000009</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000010</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000011</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000012</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000013</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000014</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000015</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000016</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000017</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000018</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000019</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000020</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000021</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000022</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000023</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534.000024</t>
-  </si>
-  <si>
-    <t>Data_20170414_121534</t>
+    <t>Data_20170712_091645.000000</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000001</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000002</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000003</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000004</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000005</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000006</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000007</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000008</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000009</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000010</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000011</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000012</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000013</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000014</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000015</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000016</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000017</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000018</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000019</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000020</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000021</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000022</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000023</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000024</t>
+  </si>
+  <si>
+    <t>Sim_Id</t>
   </si>
   <si>
     <t>Sim_Result</t>
   </si>
   <si>
-    <t>Sim_Id</t>
+    <t>Name</t>
   </si>
   <si>
     <t>Min</t>
   </si>
   <si>
     <t>Max</t>
-  </si>
-  <si>
-    <t>Name</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -195,35 +194,26 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="1" fillId="0" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle builtinId="0" hidden="0" name="Normal" xfId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium9"/>
 </styleSheet>
 </file>
 
@@ -511,16 +501,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -528,94 +522,106 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3">
+        <v>4</v>
+      </c>
+      <c r="B3" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4">
-        <v>2.25</v>
+        <v>5</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5">
-        <v>3</v>
+        <v>6</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2.25</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B6">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="B6" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7">
+        <v>8</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="n">
         <v>0.75</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F26"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="F1" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B2">
+        <v>16</v>
+      </c>
+      <c r="B2" t="n">
         <v>0</v>
       </c>
-      <c r="C2">
-        <v>-42.20761143380965</v>
-      </c>
-      <c r="D2">
-        <v>-62.46217179836616</v>
+      <c r="C2" t="n">
+        <v>42.60008858631097</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-98.3934093560363</v>
       </c>
       <c r="E2" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
@@ -623,19 +629,19 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3">
-        <v>44.36400085707389</v>
-      </c>
-      <c r="D3">
-        <v>64.28599436270147</v>
+        <v>18</v>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>12.98655752974569</v>
+      </c>
+      <c r="D3" t="n">
+        <v>-72.76295324341908</v>
       </c>
       <c r="E3" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -643,19 +649,19 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4">
+        <v>19</v>
+      </c>
+      <c r="B4" t="n">
         <v>2</v>
       </c>
-      <c r="C4">
-        <v>41.73026440160139</v>
-      </c>
-      <c r="D4">
-        <v>50.3406263634545</v>
+      <c r="C4" t="n">
+        <v>32.91979181399475</v>
+      </c>
+      <c r="D4" t="n">
+        <v>48.16203748183855</v>
       </c>
       <c r="E4" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -663,19 +669,19 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5">
+        <v>20</v>
+      </c>
+      <c r="B5" t="n">
         <v>3</v>
       </c>
-      <c r="C5">
-        <v>-12.5471371736305</v>
-      </c>
-      <c r="D5">
-        <v>-29.632201036231</v>
+      <c r="C5" t="n">
+        <v>-6.550350622651244</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-5.199952878533566</v>
       </c>
       <c r="E5" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F5" t="b">
         <v>1</v>
@@ -683,19 +689,19 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6">
+        <v>21</v>
+      </c>
+      <c r="B6" t="n">
         <v>4</v>
       </c>
-      <c r="C6">
-        <v>-31.19502837885228</v>
-      </c>
-      <c r="D6">
-        <v>-27.38540236140669</v>
+      <c r="C6" t="n">
+        <v>-31.058950132989</v>
+      </c>
+      <c r="D6" t="n">
+        <v>35.13414910098504</v>
       </c>
       <c r="E6" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
@@ -703,19 +709,19 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7">
+        <v>22</v>
+      </c>
+      <c r="B7" t="n">
         <v>5</v>
       </c>
-      <c r="C7">
-        <v>5.933996642984432</v>
-      </c>
-      <c r="D7">
-        <v>-0.6858117301123343</v>
+      <c r="C7" t="n">
+        <v>49.33460929423681</v>
+      </c>
+      <c r="D7" t="n">
+        <v>53.99749461562945</v>
       </c>
       <c r="E7" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
@@ -723,19 +729,19 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8">
+        <v>23</v>
+      </c>
+      <c r="B8" t="n">
         <v>6</v>
       </c>
-      <c r="C8">
-        <v>15.89549319968255</v>
-      </c>
-      <c r="D8">
-        <v>14.17523920316755</v>
+      <c r="C8" t="n">
+        <v>-21.81924422676842</v>
+      </c>
+      <c r="D8" t="n">
+        <v>-44.96857943583274</v>
       </c>
       <c r="E8" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F8" t="b">
         <v>1</v>
@@ -743,19 +749,19 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9">
+        <v>24</v>
+      </c>
+      <c r="B9" t="n">
         <v>7</v>
       </c>
-      <c r="C9">
-        <v>19.39717841582363</v>
-      </c>
-      <c r="D9">
-        <v>34.35274232998907</v>
+      <c r="C9" t="n">
+        <v>18.04134313372398</v>
+      </c>
+      <c r="D9" t="n">
+        <v>-66.7722427881022</v>
       </c>
       <c r="E9" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F9" t="b">
         <v>1</v>
@@ -763,19 +769,19 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10">
+        <v>25</v>
+      </c>
+      <c r="B10" t="n">
         <v>8</v>
       </c>
-      <c r="C10">
-        <v>-20.35035820926004</v>
-      </c>
-      <c r="D10">
-        <v>78.42689880326574</v>
+      <c r="C10" t="n">
+        <v>7.327514754570672</v>
+      </c>
+      <c r="D10" t="n">
+        <v>98.22724452252584</v>
       </c>
       <c r="E10" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F10" t="b">
         <v>1</v>
@@ -783,19 +789,19 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11">
+        <v>26</v>
+      </c>
+      <c r="B11" t="n">
         <v>9</v>
       </c>
-      <c r="C11">
-        <v>31.92789155401573</v>
-      </c>
-      <c r="D11">
-        <v>4.569008450293424</v>
+      <c r="C11" t="n">
+        <v>-12.08630949332292</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-24.11813681283702</v>
       </c>
       <c r="E11" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F11" t="b">
         <v>1</v>
@@ -803,19 +809,19 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B12">
+        <v>27</v>
+      </c>
+      <c r="B12" t="n">
         <v>10</v>
       </c>
-      <c r="C12">
-        <v>-0.8808073652959578</v>
-      </c>
-      <c r="D12">
-        <v>-37.73236061122333</v>
+      <c r="C12" t="n">
+        <v>-47.64771947118193</v>
+      </c>
+      <c r="D12" t="n">
+        <v>-55.88527229952129</v>
       </c>
       <c r="E12" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F12" t="b">
         <v>1</v>
@@ -823,19 +829,19 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B13">
+        <v>28</v>
+      </c>
+      <c r="B13" t="n">
         <v>11</v>
       </c>
-      <c r="C13">
-        <v>-5.716238938654286</v>
-      </c>
-      <c r="D13">
-        <v>-74.22287265852877</v>
+      <c r="C13" t="n">
+        <v>28.96434324059942</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3.039755983049247</v>
       </c>
       <c r="E13" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F13" t="b">
         <v>1</v>
@@ -843,19 +849,19 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B14">
+        <v>29</v>
+      </c>
+      <c r="B14" t="n">
         <v>12</v>
       </c>
-      <c r="C14">
-        <v>-47.95666862561361</v>
-      </c>
-      <c r="D14">
-        <v>-93.33860738482592</v>
+      <c r="C14" t="n">
+        <v>-27.56569228945906</v>
+      </c>
+      <c r="D14" t="n">
+        <v>26.77552914956441</v>
       </c>
       <c r="E14" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F14" t="b">
         <v>1</v>
@@ -863,19 +869,19 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15">
+        <v>30</v>
+      </c>
+      <c r="B15" t="n">
         <v>13</v>
       </c>
-      <c r="C15">
-        <v>36.49020575380368</v>
-      </c>
-      <c r="D15">
-        <v>59.45839102994054</v>
+      <c r="C15" t="n">
+        <v>-22.77114703949607</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-36.61337421158958</v>
       </c>
       <c r="E15" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F15" t="b">
         <v>1</v>
@@ -883,19 +889,19 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B16">
+        <v>31</v>
+      </c>
+      <c r="B16" t="n">
         <v>14</v>
       </c>
-      <c r="C16">
-        <v>24.85831826755167</v>
-      </c>
-      <c r="D16">
-        <v>86.36912834690719</v>
+      <c r="C16" t="n">
+        <v>24.3224863606699</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-29.11475831121508</v>
       </c>
       <c r="E16" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F16" t="b">
         <v>1</v>
@@ -903,19 +909,19 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B17">
+        <v>32</v>
+      </c>
+      <c r="B17" t="n">
         <v>15</v>
       </c>
-      <c r="C17">
-        <v>7.4647980155328</v>
-      </c>
-      <c r="D17">
-        <v>-8.967576458363183</v>
+      <c r="C17" t="n">
+        <v>-5.402572267828766</v>
+      </c>
+      <c r="D17" t="n">
+        <v>91.32934791741965</v>
       </c>
       <c r="E17" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F17" t="b">
         <v>1</v>
@@ -923,19 +929,19 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B18">
+        <v>33</v>
+      </c>
+      <c r="B18" t="n">
         <v>16</v>
       </c>
-      <c r="C18">
-        <v>-36.8068677966816</v>
-      </c>
-      <c r="D18">
-        <v>41.83528392737512</v>
+      <c r="C18" t="n">
+        <v>-40.67115771967745</v>
+      </c>
+      <c r="D18" t="n">
+        <v>-87.53396823192645</v>
       </c>
       <c r="E18" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F18" t="b">
         <v>1</v>
@@ -943,19 +949,19 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B19">
-        <v>17</v>
-      </c>
-      <c r="C19">
-        <v>-9.965982424035488</v>
-      </c>
-      <c r="D19">
-        <v>92.81856890601051</v>
+        <v>34</v>
+      </c>
+      <c r="B19" t="n">
+        <v>17</v>
+      </c>
+      <c r="C19" t="n">
+        <v>-0.4368505723745884</v>
+      </c>
+      <c r="D19" t="n">
+        <v>9.432466320620222</v>
       </c>
       <c r="E19" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F19" t="b">
         <v>1</v>
@@ -963,19 +969,19 @@
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B20">
+        <v>35</v>
+      </c>
+      <c r="B20" t="n">
         <v>18</v>
       </c>
-      <c r="C20">
-        <v>28.26976625774897</v>
-      </c>
-      <c r="D20">
-        <v>-13.39100428734896</v>
+      <c r="C20" t="n">
+        <v>-16.72196598646099</v>
+      </c>
+      <c r="D20" t="n">
+        <v>43.45888310351546</v>
       </c>
       <c r="E20" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F20" t="b">
         <v>0</v>
@@ -983,19 +989,19 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B21">
+        <v>36</v>
+      </c>
+      <c r="B21" t="n">
         <v>19</v>
       </c>
-      <c r="C21">
-        <v>-27.74881279709197</v>
-      </c>
-      <c r="D21">
-        <v>-48.54208872705258</v>
+      <c r="C21" t="n">
+        <v>15.29634713476852</v>
+      </c>
+      <c r="D21" t="n">
+        <v>-83.04313422864848</v>
       </c>
       <c r="E21" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F21" t="b">
         <v>0</v>
@@ -1003,19 +1009,19 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B22">
+        <v>37</v>
+      </c>
+      <c r="B22" t="n">
         <v>20</v>
       </c>
-      <c r="C22">
-        <v>-14.90323808547211</v>
-      </c>
-      <c r="D22">
-        <v>73.42646483762144</v>
+      <c r="C22" t="n">
+        <v>37.01032927000048</v>
+      </c>
+      <c r="D22" t="n">
+        <v>14.28531620098244</v>
       </c>
       <c r="E22" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F22" t="b">
         <v>0</v>
@@ -1023,19 +1029,19 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B23">
+        <v>38</v>
+      </c>
+      <c r="B23" t="n">
         <v>21</v>
       </c>
-      <c r="C23">
-        <v>-41.44127180358139</v>
-      </c>
-      <c r="D23">
-        <v>-55.80511911935229</v>
+      <c r="C23" t="n">
+        <v>5.831376134756006</v>
+      </c>
+      <c r="D23" t="n">
+        <v>-14.57852141958386</v>
       </c>
       <c r="E23" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F23" t="b">
         <v>0</v>
@@ -1043,19 +1049,19 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B24">
+        <v>39</v>
+      </c>
+      <c r="B24" t="n">
         <v>22</v>
       </c>
-      <c r="C24">
-        <v>10.98188747733819</v>
-      </c>
-      <c r="D24">
-        <v>26.91239022115901</v>
+      <c r="C24" t="n">
+        <v>41.12394811855083</v>
+      </c>
+      <c r="D24" t="n">
+        <v>60.41378758903392</v>
       </c>
       <c r="E24" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F24" t="b">
         <v>0</v>
@@ -1063,19 +1069,19 @@
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B25">
+        <v>40</v>
+      </c>
+      <c r="B25" t="n">
         <v>23</v>
       </c>
-      <c r="C25">
-        <v>-25.01688191022813</v>
-      </c>
-      <c r="D25">
-        <v>-85.8779545656617</v>
+      <c r="C25" t="n">
+        <v>-44.89685426926108</v>
+      </c>
+      <c r="D25" t="n">
+        <v>72.48911130599336</v>
       </c>
       <c r="E25" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F25" t="b">
         <v>0</v>
@@ -1083,520 +1089,528 @@
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="B26">
+        <v>41</v>
+      </c>
+      <c r="B26" t="n">
         <v>24</v>
       </c>
-      <c r="C26">
-        <v>49.00305676792436</v>
-      </c>
-      <c r="D26">
-        <v>-81.46904140852911</v>
+      <c r="C26" t="n">
+        <v>-34.31380334221465</v>
+      </c>
+      <c r="D26" t="n">
+        <v>80.36361379626152</v>
       </c>
       <c r="E26" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="F26" t="b">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E26"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="C1" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>42</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C2" s="1">
+        <v>17</v>
+      </c>
+      <c r="C2" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="E2">
-        <v>76.19355676105398</v>
+      <c r="E2" t="n">
+        <v>106.5456748982687</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C3" s="1">
-        <v>1</v>
-      </c>
-      <c r="D3" s="1">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>76.36690026547718</v>
+        <v>17</v>
+      </c>
+      <c r="C3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>73.89752703384607</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C4" s="1">
+        <v>17</v>
+      </c>
+      <c r="C4" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E4">
-        <v>67.14850693117126</v>
+      <c r="E4" t="n">
+        <v>57.92193386035419</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C5" s="1">
+        <v>17</v>
+      </c>
+      <c r="C5" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E5">
-        <v>31.48450554964168</v>
+      <c r="E5" t="n">
+        <v>6.802317084858752</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C6" s="1">
+        <v>17</v>
+      </c>
+      <c r="C6" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="E6">
-        <v>41.7230888751962</v>
+      <c r="E6" t="n">
+        <v>46.31010965981822</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C7" s="1">
+        <v>17</v>
+      </c>
+      <c r="C7" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="E7">
-        <v>4.37557979269938</v>
+      <c r="E7" t="n">
+        <v>73.10443797153236</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8" s="1">
+        <v>17</v>
+      </c>
+      <c r="C8" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="E8">
-        <v>20.31912770952653</v>
+      <c r="E8" t="n">
+        <v>49.38195201450795</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" s="1">
+        <v>17</v>
+      </c>
+      <c r="C9" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="E9">
-        <v>39.8990125763121</v>
+      <c r="E9" t="n">
+        <v>69.98570443035528</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C10" s="1">
+        <v>17</v>
+      </c>
+      <c r="C10" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D10" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="E10">
-        <v>80.99236102485536</v>
+      <c r="E10" t="n">
+        <v>98.62043964575052</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" s="1">
+        <v>17</v>
+      </c>
+      <c r="C11" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="D11" s="1">
+      <c r="D11" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="E11">
-        <v>32.20960179272636</v>
+      <c r="E11" t="n">
+        <v>27.53711867095363</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" s="1">
+        <v>17</v>
+      </c>
+      <c r="C12" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="E12">
-        <v>37.53822042356747</v>
+      <c r="E12" t="n">
+        <v>76.0357221648465</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" s="1">
+        <v>17</v>
+      </c>
+      <c r="C13" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="E13">
-        <v>73.83721255468465</v>
+      <c r="E13" t="n">
+        <v>29.66757213645581</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" s="1">
+        <v>17</v>
+      </c>
+      <c r="C14" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="E14">
-        <v>104.7949303011075</v>
+      <c r="E14" t="n">
+        <v>39.12139459322662</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C15" s="1">
+        <v>17</v>
+      </c>
+      <c r="C15" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D15" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="E15">
-        <v>68.62015993190829</v>
+      <c r="E15" t="n">
+        <v>42.07181497767856</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C16" s="1">
+        <v>17</v>
+      </c>
+      <c r="C16" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="E16">
-        <v>87.68275321799192</v>
+      <c r="E16" t="n">
+        <v>39.36598465453883</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C17" s="1">
+        <v>17</v>
+      </c>
+      <c r="C17" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="E17">
-        <v>10.80369943174134</v>
+      <c r="E17" t="n">
+        <v>91.08311917838569</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C18" s="1">
+        <v>17</v>
+      </c>
+      <c r="C18" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="E18">
-        <v>55.18649259927105</v>
+      <c r="E18" t="n">
+        <v>97.02142426461921</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C19" s="1">
-        <v>17</v>
-      </c>
-      <c r="D19" s="1">
-        <v>17</v>
-      </c>
-      <c r="E19">
-        <v>92.8813400088017</v>
+        <v>17</v>
+      </c>
+      <c r="C19" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="D19" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="E19" t="n">
+        <v>9.645929068109689</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C20" s="1">
+        <v>17</v>
+      </c>
+      <c r="C20" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="E20">
-        <v>30.38395706671946</v>
+      <c r="E20" t="n">
+        <v>46.39499843045764</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C21" s="1">
+        <v>17</v>
+      </c>
+      <c r="C21" s="1" t="n">
         <v>19</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21" s="1" t="n">
         <v>19</v>
       </c>
-      <c r="E21">
-        <v>55.82677758100662</v>
+      <c r="E21" t="n">
+        <v>84.06699852812513</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C22" s="1">
+        <v>17</v>
+      </c>
+      <c r="C22" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="D22" s="1">
+      <c r="D22" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="E22">
-        <v>73.71241013447565</v>
+      <c r="E22" t="n">
+        <v>39.3699828767349</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C23" s="1">
+        <v>17</v>
+      </c>
+      <c r="C23" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="D23" s="1">
+      <c r="D23" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="E23">
-        <v>70.67363370791277</v>
+      <c r="E23" t="n">
+        <v>15.08660231552476</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C24" s="1">
+        <v>17</v>
+      </c>
+      <c r="C24" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="D24" s="1">
+      <c r="D24" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="E24">
-        <v>28.51923253562785</v>
+      <c r="E24" t="n">
+        <v>72.64484137651345</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C25" s="1">
+        <v>17</v>
+      </c>
+      <c r="C25" s="1" t="n">
         <v>23</v>
       </c>
-      <c r="D25" s="1">
+      <c r="D25" s="1" t="n">
         <v>23</v>
       </c>
-      <c r="E25">
-        <v>89.30281350114838</v>
+      <c r="E25" t="n">
+        <v>86.09220555690713</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C26" s="1">
+        <v>17</v>
+      </c>
+      <c r="C26" s="1" t="n">
         <v>24</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26" s="1" t="n">
         <v>24</v>
       </c>
-      <c r="E26">
-        <v>95.11454358416995</v>
+      <c r="E26" t="n">
+        <v>87.90710633663716</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>43</v>
-      </c>
       <c r="C1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2">
+        <v>12</v>
+      </c>
+      <c r="B2" t="n">
         <v>-50</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3">
+        <v>13</v>
+      </c>
+      <c r="B3" t="n">
         <v>-100</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="n">
         <v>100</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Working towards python 3 compatibility
</commit_message>
<xml_diff>
--- a/history_matching/example/iter0/Cuts/RadiusShouldBe15/history_matching_config.xlsx
+++ b/history_matching/example/iter0/Cuts/RadiusShouldBe15/history_matching_config.xlsx
@@ -2,6 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
     <workbookView activeTab="0"/>
   </bookViews>
@@ -67,82 +68,82 @@
     <t>Train</t>
   </si>
   <si>
-    <t>Data_20170712_091645.000000</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000001</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000002</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000003</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000004</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000005</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000006</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000007</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000008</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000009</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000010</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000011</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000012</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000013</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000014</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000015</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000016</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000017</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000018</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000019</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000020</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000021</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000022</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000023</t>
-  </si>
-  <si>
-    <t>Data_20170712_091645.000024</t>
+    <t>Data_20180119_001620.000000</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000001</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000002</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000003</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000004</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000005</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000006</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000007</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000008</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000009</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000010</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000011</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000012</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000013</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000014</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000015</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000016</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000017</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000018</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000019</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000020</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000021</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000022</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000023</t>
+  </si>
+  <si>
+    <t>Data_20180119_001620.000024</t>
   </si>
   <si>
     <t>Sim_Id</t>
@@ -615,10 +616,10 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>42.60008858631097</v>
+        <v>36.97383846810624</v>
       </c>
       <c r="D2" t="n">
-        <v>-98.3934093560363</v>
+        <v>96.6067982109376</v>
       </c>
       <c r="E2" t="s">
         <v>17</v>
@@ -635,10 +636,10 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>12.98655752974569</v>
+        <v>-47.59430216678409</v>
       </c>
       <c r="D3" t="n">
-        <v>-72.76295324341908</v>
+        <v>41.94953896263729</v>
       </c>
       <c r="E3" t="s">
         <v>17</v>
@@ -655,10 +656,10 @@
         <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>32.91979181399475</v>
+        <v>23.67099048551562</v>
       </c>
       <c r="D4" t="n">
-        <v>48.16203748183855</v>
+        <v>66.58932634912242</v>
       </c>
       <c r="E4" t="s">
         <v>17</v>
@@ -675,10 +676,10 @@
         <v>3</v>
       </c>
       <c r="C5" t="n">
-        <v>-6.550350622651244</v>
+        <v>-32.12690480729383</v>
       </c>
       <c r="D5" t="n">
-        <v>-5.199952878533566</v>
+        <v>-95.12935873795897</v>
       </c>
       <c r="E5" t="s">
         <v>17</v>
@@ -695,10 +696,10 @@
         <v>4</v>
       </c>
       <c r="C6" t="n">
-        <v>-31.058950132989</v>
+        <v>33.06948879076657</v>
       </c>
       <c r="D6" t="n">
-        <v>35.13414910098504</v>
+        <v>78.58966428484089</v>
       </c>
       <c r="E6" t="s">
         <v>17</v>
@@ -715,10 +716,10 @@
         <v>5</v>
       </c>
       <c r="C7" t="n">
-        <v>49.33460929423681</v>
+        <v>-21.54393314536323</v>
       </c>
       <c r="D7" t="n">
-        <v>53.99749461562945</v>
+        <v>-73.27452020965829</v>
       </c>
       <c r="E7" t="s">
         <v>17</v>
@@ -735,10 +736,10 @@
         <v>6</v>
       </c>
       <c r="C8" t="n">
-        <v>-21.81924422676842</v>
+        <v>-28.70199886941015</v>
       </c>
       <c r="D8" t="n">
-        <v>-44.96857943583274</v>
+        <v>-5.028730151675362</v>
       </c>
       <c r="E8" t="s">
         <v>17</v>
@@ -755,10 +756,10 @@
         <v>7</v>
       </c>
       <c r="C9" t="n">
-        <v>18.04134313372398</v>
+        <v>-1.744167862823204</v>
       </c>
       <c r="D9" t="n">
-        <v>-66.7722427881022</v>
+        <v>55.33128222122482</v>
       </c>
       <c r="E9" t="s">
         <v>17</v>
@@ -775,10 +776,10 @@
         <v>8</v>
       </c>
       <c r="C10" t="n">
-        <v>7.327514754570672</v>
+        <v>-14.28831588713167</v>
       </c>
       <c r="D10" t="n">
-        <v>98.22724452252584</v>
+        <v>-45.94463204277744</v>
       </c>
       <c r="E10" t="s">
         <v>17</v>
@@ -795,10 +796,10 @@
         <v>9</v>
       </c>
       <c r="C11" t="n">
-        <v>-12.08630949332292</v>
+        <v>49.64962080146476</v>
       </c>
       <c r="D11" t="n">
-        <v>-24.11813681283702</v>
+        <v>-56.14936736637327</v>
       </c>
       <c r="E11" t="s">
         <v>17</v>
@@ -815,10 +816,10 @@
         <v>10</v>
       </c>
       <c r="C12" t="n">
-        <v>-47.64771947118193</v>
+        <v>-37.48296455355791</v>
       </c>
       <c r="D12" t="n">
-        <v>-55.88527229952129</v>
+        <v>-25.35359443624601</v>
       </c>
       <c r="E12" t="s">
         <v>17</v>
@@ -835,10 +836,10 @@
         <v>11</v>
       </c>
       <c r="C13" t="n">
-        <v>28.96434324059942</v>
+        <v>7.71449199266803</v>
       </c>
       <c r="D13" t="n">
-        <v>3.039755983049247</v>
+        <v>9.458312247592588</v>
       </c>
       <c r="E13" t="s">
         <v>17</v>
@@ -855,10 +856,10 @@
         <v>12</v>
       </c>
       <c r="C14" t="n">
-        <v>-27.56569228945906</v>
+        <v>40.63332465138902</v>
       </c>
       <c r="D14" t="n">
-        <v>26.77552914956441</v>
+        <v>32.88548096077622</v>
       </c>
       <c r="E14" t="s">
         <v>17</v>
@@ -875,10 +876,10 @@
         <v>13</v>
       </c>
       <c r="C15" t="n">
-        <v>-22.77114703949607</v>
+        <v>-2.447090783119101</v>
       </c>
       <c r="D15" t="n">
-        <v>-36.61337421158958</v>
+        <v>2.591343404656541</v>
       </c>
       <c r="E15" t="s">
         <v>17</v>
@@ -895,10 +896,10 @@
         <v>14</v>
       </c>
       <c r="C16" t="n">
-        <v>24.3224863606699</v>
+        <v>-39.91611073298978</v>
       </c>
       <c r="D16" t="n">
-        <v>-29.11475831121508</v>
+        <v>-89.59025782321442</v>
       </c>
       <c r="E16" t="s">
         <v>17</v>
@@ -915,10 +916,10 @@
         <v>15</v>
       </c>
       <c r="C17" t="n">
-        <v>-5.402572267828766</v>
+        <v>-13.6059741872424</v>
       </c>
       <c r="D17" t="n">
-        <v>91.32934791741965</v>
+        <v>87.43968560451231</v>
       </c>
       <c r="E17" t="s">
         <v>17</v>
@@ -935,10 +936,10 @@
         <v>16</v>
       </c>
       <c r="C18" t="n">
-        <v>-40.67115771967745</v>
+        <v>-9.10312145162537</v>
       </c>
       <c r="D18" t="n">
-        <v>-87.53396823192645</v>
+        <v>13.59593024948138</v>
       </c>
       <c r="E18" t="s">
         <v>17</v>
@@ -955,10 +956,10 @@
         <v>17</v>
       </c>
       <c r="C19" t="n">
-        <v>-0.4368505723745884</v>
+        <v>26.17179564370285</v>
       </c>
       <c r="D19" t="n">
-        <v>9.432466320620222</v>
+        <v>-35.76449135823198</v>
       </c>
       <c r="E19" t="s">
         <v>17</v>
@@ -975,10 +976,10 @@
         <v>18</v>
       </c>
       <c r="C20" t="n">
-        <v>-16.72196598646099</v>
+        <v>3.548724135704674</v>
       </c>
       <c r="D20" t="n">
-        <v>43.45888310351546</v>
+        <v>-37.01012112572288</v>
       </c>
       <c r="E20" t="s">
         <v>17</v>
@@ -995,10 +996,10 @@
         <v>19</v>
       </c>
       <c r="C21" t="n">
-        <v>15.29634713476852</v>
+        <v>-45.72639341354221</v>
       </c>
       <c r="D21" t="n">
-        <v>-83.04313422864848</v>
+        <v>-64.60699725731783</v>
       </c>
       <c r="E21" t="s">
         <v>17</v>
@@ -1015,10 +1016,10 @@
         <v>20</v>
       </c>
       <c r="C22" t="n">
-        <v>37.01032927000048</v>
+        <v>15.47473036233153</v>
       </c>
       <c r="D22" t="n">
-        <v>14.28531620098244</v>
+        <v>-19.07164464498223</v>
       </c>
       <c r="E22" t="s">
         <v>17</v>
@@ -1035,10 +1036,10 @@
         <v>21</v>
       </c>
       <c r="C23" t="n">
-        <v>5.831376134756006</v>
+        <v>42.19946580172682</v>
       </c>
       <c r="D23" t="n">
-        <v>-14.57852141958386</v>
+        <v>74.16432818162795</v>
       </c>
       <c r="E23" t="s">
         <v>17</v>
@@ -1055,10 +1056,10 @@
         <v>22</v>
       </c>
       <c r="C24" t="n">
-        <v>41.12394811855083</v>
+        <v>11.36092669010599</v>
       </c>
       <c r="D24" t="n">
-        <v>60.41378758903392</v>
+        <v>-76.26939573709377</v>
       </c>
       <c r="E24" t="s">
         <v>17</v>
@@ -1075,10 +1076,10 @@
         <v>23</v>
       </c>
       <c r="C25" t="n">
-        <v>-44.89685426926108</v>
+        <v>-24.82091293894687</v>
       </c>
       <c r="D25" t="n">
-        <v>72.48911130599336</v>
+        <v>49.83916472955462</v>
       </c>
       <c r="E25" t="s">
         <v>17</v>
@@ -1095,10 +1096,10 @@
         <v>24</v>
       </c>
       <c r="C26" t="n">
-        <v>-34.31380334221465</v>
+        <v>18.37217291828543</v>
       </c>
       <c r="D26" t="n">
-        <v>80.36361379626152</v>
+        <v>24.80290404671575</v>
       </c>
       <c r="E26" t="s">
         <v>17</v>
@@ -1152,7 +1153,7 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>106.5456748982687</v>
+        <v>104.5829775889917</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1169,7 +1170,7 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>73.89752703384607</v>
+        <v>61.9654847667875</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1186,7 +1187,7 @@
         <v>2</v>
       </c>
       <c r="E4" t="n">
-        <v>57.92193386035419</v>
+        <v>71.00834208927171</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -1203,7 +1204,7 @@
         <v>3</v>
       </c>
       <c r="E5" t="n">
-        <v>6.802317084858752</v>
+        <v>102.1323052223888</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -1220,7 +1221,7 @@
         <v>4</v>
       </c>
       <c r="E6" t="n">
-        <v>46.31010965981822</v>
+        <v>85.12384449268366</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -1237,7 +1238,7 @@
         <v>5</v>
       </c>
       <c r="E7" t="n">
-        <v>73.10443797153236</v>
+        <v>77.51395401914888</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -1254,7 +1255,7 @@
         <v>6</v>
       </c>
       <c r="E8" t="n">
-        <v>49.38195201450795</v>
+        <v>28.92244249308711</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -1271,7 +1272,7 @@
         <v>7</v>
       </c>
       <c r="E9" t="n">
-        <v>69.98570443035528</v>
+        <v>57.19828906317157</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -1288,7 +1289,7 @@
         <v>8</v>
       </c>
       <c r="E10" t="n">
-        <v>98.62043964575052</v>
+        <v>48.9199220671023</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -1305,7 +1306,7 @@
         <v>9</v>
       </c>
       <c r="E11" t="n">
-        <v>27.53711867095363</v>
+        <v>75.33121099590072</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -1322,7 +1323,7 @@
         <v>10</v>
       </c>
       <c r="E12" t="n">
-        <v>76.0357221648465</v>
+        <v>46.0612601290569</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -1339,7 +1340,7 @@
         <v>11</v>
       </c>
       <c r="E13" t="n">
-        <v>29.66757213645581</v>
+        <v>11.86042758978058</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -1356,7 +1357,7 @@
         <v>12</v>
       </c>
       <c r="E14" t="n">
-        <v>39.12139459322662</v>
+        <v>52.77480993080396</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -1373,7 +1374,7 @@
         <v>13</v>
       </c>
       <c r="E15" t="n">
-        <v>42.07181497767856</v>
+        <v>2.712014305147573</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -1390,7 +1391,7 @@
         <v>14</v>
       </c>
       <c r="E16" t="n">
-        <v>39.36598465453883</v>
+        <v>98.71819265777106</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -1407,7 +1408,7 @@
         <v>15</v>
       </c>
       <c r="E17" t="n">
-        <v>91.08311917838569</v>
+        <v>88.29274435448015</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -1424,7 +1425,7 @@
         <v>16</v>
       </c>
       <c r="E18" t="n">
-        <v>97.02142426461921</v>
+        <v>16.65599440954206</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -1441,7 +1442,7 @@
         <v>17</v>
       </c>
       <c r="E19" t="n">
-        <v>9.645929068109689</v>
+        <v>43.63750166270777</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -1458,7 +1459,7 @@
         <v>18</v>
       </c>
       <c r="E20" t="n">
-        <v>46.39499843045764</v>
+        <v>35.46164363756871</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -1475,7 +1476,7 @@
         <v>19</v>
       </c>
       <c r="E21" t="n">
-        <v>84.06699852812513</v>
+        <v>80.89494868450986</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -1492,7 +1493,7 @@
         <v>20</v>
       </c>
       <c r="E22" t="n">
-        <v>39.3699828767349</v>
+        <v>24.2314259715583</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -1509,7 +1510,7 @@
         <v>21</v>
       </c>
       <c r="E23" t="n">
-        <v>15.08660231552476</v>
+        <v>86.68066924689877</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -1526,7 +1527,7 @@
         <v>22</v>
       </c>
       <c r="E24" t="n">
-        <v>72.64484137651345</v>
+        <v>77.78161804821913</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -1543,7 +1544,7 @@
         <v>23</v>
       </c>
       <c r="E25" t="n">
-        <v>86.09220555690713</v>
+        <v>55.52592106354519</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -1560,7 +1561,7 @@
         <v>24</v>
       </c>
       <c r="E26" t="n">
-        <v>87.90710633663716</v>
+        <v>30.88798407885472</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Further progress towards python 3
</commit_message>
<xml_diff>
--- a/history_matching/example/iter0/Cuts/RadiusShouldBe15/history_matching_config.xlsx
+++ b/history_matching/example/iter0/Cuts/RadiusShouldBe15/history_matching_config.xlsx
@@ -1119,448 +1119,292 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>14</v>
+        <v>42</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E1" s="1" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" s="1" t="n">
+      <c r="B2" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="n">
+      <c r="C2" t="n">
         <v>104.5829775889917</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" t="n">
+      <c r="B3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
         <v>61.9654847667875</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="1" t="n">
+      <c r="B4" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D4" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E4" t="n">
+      <c r="C4" t="n">
         <v>71.00834208927171</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:3">
       <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="1" t="n">
+      <c r="B5" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="E5" t="n">
+      <c r="C5" t="n">
         <v>102.1323052223888</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="1" t="n">
+      <c r="B6" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D6" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E6" t="n">
+      <c r="C6" t="n">
         <v>85.12384449268366</v>
       </c>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:3">
       <c r="A7" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="1" t="n">
+      <c r="B7" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D7" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="E7" t="n">
+      <c r="C7" t="n">
         <v>77.51395401914888</v>
       </c>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:3">
       <c r="A8" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="1" t="n">
+      <c r="B8" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D8" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="E8" t="n">
+      <c r="C8" t="n">
         <v>28.92244249308711</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:3">
       <c r="A9" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="1" t="n">
+      <c r="B9" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="D9" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="E9" t="n">
+      <c r="C9" t="n">
         <v>57.19828906317157</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:3">
       <c r="A10" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="1" t="n">
+      <c r="B10" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="D10" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="E10" t="n">
+      <c r="C10" t="n">
         <v>48.9199220671023</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:3">
       <c r="A11" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" s="1" t="n">
+      <c r="B11" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="D11" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="E11" t="n">
+      <c r="C11" t="n">
         <v>75.33121099590072</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:3">
       <c r="A12" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" s="1" t="n">
+      <c r="B12" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="D12" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="E12" t="n">
+      <c r="C12" t="n">
         <v>46.0612601290569</v>
       </c>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:3">
       <c r="A13" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="1" t="n">
+      <c r="B13" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="D13" s="1" t="n">
-        <v>11</v>
-      </c>
-      <c r="E13" t="n">
+      <c r="C13" t="n">
         <v>11.86042758978058</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:3">
       <c r="A14" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C14" s="1" t="n">
+      <c r="B14" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="D14" s="1" t="n">
-        <v>12</v>
-      </c>
-      <c r="E14" t="n">
+      <c r="C14" t="n">
         <v>52.77480993080396</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:3">
       <c r="A15" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C15" s="1" t="n">
+      <c r="B15" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="D15" s="1" t="n">
-        <v>13</v>
-      </c>
-      <c r="E15" t="n">
+      <c r="C15" t="n">
         <v>2.712014305147573</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:3">
       <c r="A16" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16" s="1" t="n">
+      <c r="B16" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="D16" s="1" t="n">
-        <v>14</v>
-      </c>
-      <c r="E16" t="n">
+      <c r="C16" t="n">
         <v>98.71819265777106</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:3">
       <c r="A17" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C17" s="1" t="n">
+      <c r="B17" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="D17" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="E17" t="n">
+      <c r="C17" t="n">
         <v>88.29274435448015</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:3">
       <c r="A18" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C18" s="1" t="n">
+      <c r="B18" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="D18" s="1" t="n">
-        <v>16</v>
-      </c>
-      <c r="E18" t="n">
+      <c r="C18" t="n">
         <v>16.65599440954206</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:3">
       <c r="A19" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C19" s="1" t="n">
-        <v>17</v>
-      </c>
-      <c r="D19" s="1" t="n">
-        <v>17</v>
-      </c>
-      <c r="E19" t="n">
+      <c r="B19" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="C19" t="n">
         <v>43.63750166270777</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:3">
       <c r="A20" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C20" s="1" t="n">
+      <c r="B20" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="D20" s="1" t="n">
-        <v>18</v>
-      </c>
-      <c r="E20" t="n">
+      <c r="C20" t="n">
         <v>35.46164363756871</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:3">
       <c r="A21" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B21" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C21" s="1" t="n">
+      <c r="B21" s="1" t="n">
         <v>19</v>
       </c>
-      <c r="D21" s="1" t="n">
-        <v>19</v>
-      </c>
-      <c r="E21" t="n">
+      <c r="C21" t="n">
         <v>80.89494868450986</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:3">
       <c r="A22" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C22" s="1" t="n">
+      <c r="B22" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="D22" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="E22" t="n">
+      <c r="C22" t="n">
         <v>24.2314259715583</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:3">
       <c r="A23" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C23" s="1" t="n">
+      <c r="B23" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="D23" s="1" t="n">
-        <v>21</v>
-      </c>
-      <c r="E23" t="n">
+      <c r="C23" t="n">
         <v>86.68066924689877</v>
       </c>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:3">
       <c r="A24" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C24" s="1" t="n">
+      <c r="B24" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="D24" s="1" t="n">
-        <v>22</v>
-      </c>
-      <c r="E24" t="n">
+      <c r="C24" t="n">
         <v>77.78161804821913</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:3">
       <c r="A25" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C25" s="1" t="n">
+      <c r="B25" s="1" t="n">
         <v>23</v>
       </c>
-      <c r="D25" s="1" t="n">
-        <v>23</v>
-      </c>
-      <c r="E25" t="n">
+      <c r="C25" t="n">
         <v>55.52592106354519</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:3">
       <c r="A26" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C26" s="1" t="n">
+      <c r="B26" s="1" t="n">
         <v>24</v>
       </c>
-      <c r="D26" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="E26" t="n">
+      <c r="C26" t="n">
         <v>30.88798407885472</v>
       </c>
     </row>

</xml_diff>

<commit_message>
All seems good, fixed a small plotting bug and tried with GPU on Linux.
</commit_message>
<xml_diff>
--- a/history_matching/example/iter0/Cuts/RadiusShouldBe15/history_matching_config.xlsx
+++ b/history_matching/example/iter0/Cuts/RadiusShouldBe15/history_matching_config.xlsx
@@ -68,82 +68,82 @@
     <t>Train</t>
   </si>
   <si>
-    <t>Data_20180119_001620.000000</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000001</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000002</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000003</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000004</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000005</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000006</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000007</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000008</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000009</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000010</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000011</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000012</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000013</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000014</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000015</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000016</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000017</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000018</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000019</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000020</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000021</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000022</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000023</t>
-  </si>
-  <si>
-    <t>Data_20180119_001620.000024</t>
+    <t>Data_20170712_091645.000000</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000001</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000002</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000003</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000004</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000005</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000006</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000007</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000008</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000009</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000010</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000011</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000012</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000013</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000014</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000015</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000016</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000017</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000018</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000019</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000020</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000021</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000022</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000023</t>
+  </si>
+  <si>
+    <t>Data_20170712_091645.000024</t>
   </si>
   <si>
     <t>Sim_Id</t>
@@ -616,10 +616,10 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>36.97383846810624</v>
+        <v>42.60008858631097</v>
       </c>
       <c r="D2" t="n">
-        <v>96.6067982109376</v>
+        <v>-98.3934093560363</v>
       </c>
       <c r="E2" t="s">
         <v>17</v>
@@ -636,10 +636,10 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>-47.59430216678409</v>
+        <v>12.98655752974569</v>
       </c>
       <c r="D3" t="n">
-        <v>41.94953896263729</v>
+        <v>-72.76295324341908</v>
       </c>
       <c r="E3" t="s">
         <v>17</v>
@@ -656,10 +656,10 @@
         <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>23.67099048551562</v>
+        <v>32.91979181399475</v>
       </c>
       <c r="D4" t="n">
-        <v>66.58932634912242</v>
+        <v>48.16203748183855</v>
       </c>
       <c r="E4" t="s">
         <v>17</v>
@@ -676,10 +676,10 @@
         <v>3</v>
       </c>
       <c r="C5" t="n">
-        <v>-32.12690480729383</v>
+        <v>-6.550350622651244</v>
       </c>
       <c r="D5" t="n">
-        <v>-95.12935873795897</v>
+        <v>-5.199952878533566</v>
       </c>
       <c r="E5" t="s">
         <v>17</v>
@@ -696,10 +696,10 @@
         <v>4</v>
       </c>
       <c r="C6" t="n">
-        <v>33.06948879076657</v>
+        <v>-31.058950132989</v>
       </c>
       <c r="D6" t="n">
-        <v>78.58966428484089</v>
+        <v>35.13414910098504</v>
       </c>
       <c r="E6" t="s">
         <v>17</v>
@@ -716,10 +716,10 @@
         <v>5</v>
       </c>
       <c r="C7" t="n">
-        <v>-21.54393314536323</v>
+        <v>49.33460929423681</v>
       </c>
       <c r="D7" t="n">
-        <v>-73.27452020965829</v>
+        <v>53.99749461562945</v>
       </c>
       <c r="E7" t="s">
         <v>17</v>
@@ -736,10 +736,10 @@
         <v>6</v>
       </c>
       <c r="C8" t="n">
-        <v>-28.70199886941015</v>
+        <v>-21.81924422676842</v>
       </c>
       <c r="D8" t="n">
-        <v>-5.028730151675362</v>
+        <v>-44.96857943583274</v>
       </c>
       <c r="E8" t="s">
         <v>17</v>
@@ -756,10 +756,10 @@
         <v>7</v>
       </c>
       <c r="C9" t="n">
-        <v>-1.744167862823204</v>
+        <v>18.04134313372398</v>
       </c>
       <c r="D9" t="n">
-        <v>55.33128222122482</v>
+        <v>-66.7722427881022</v>
       </c>
       <c r="E9" t="s">
         <v>17</v>
@@ -776,10 +776,10 @@
         <v>8</v>
       </c>
       <c r="C10" t="n">
-        <v>-14.28831588713167</v>
+        <v>7.327514754570672</v>
       </c>
       <c r="D10" t="n">
-        <v>-45.94463204277744</v>
+        <v>98.22724452252584</v>
       </c>
       <c r="E10" t="s">
         <v>17</v>
@@ -796,10 +796,10 @@
         <v>9</v>
       </c>
       <c r="C11" t="n">
-        <v>49.64962080146476</v>
+        <v>-12.08630949332292</v>
       </c>
       <c r="D11" t="n">
-        <v>-56.14936736637327</v>
+        <v>-24.11813681283702</v>
       </c>
       <c r="E11" t="s">
         <v>17</v>
@@ -816,10 +816,10 @@
         <v>10</v>
       </c>
       <c r="C12" t="n">
-        <v>-37.48296455355791</v>
+        <v>-47.64771947118193</v>
       </c>
       <c r="D12" t="n">
-        <v>-25.35359443624601</v>
+        <v>-55.88527229952129</v>
       </c>
       <c r="E12" t="s">
         <v>17</v>
@@ -836,10 +836,10 @@
         <v>11</v>
       </c>
       <c r="C13" t="n">
-        <v>7.71449199266803</v>
+        <v>28.96434324059942</v>
       </c>
       <c r="D13" t="n">
-        <v>9.458312247592588</v>
+        <v>3.039755983049247</v>
       </c>
       <c r="E13" t="s">
         <v>17</v>
@@ -856,10 +856,10 @@
         <v>12</v>
       </c>
       <c r="C14" t="n">
-        <v>40.63332465138902</v>
+        <v>-27.56569228945906</v>
       </c>
       <c r="D14" t="n">
-        <v>32.88548096077622</v>
+        <v>26.77552914956441</v>
       </c>
       <c r="E14" t="s">
         <v>17</v>
@@ -876,10 +876,10 @@
         <v>13</v>
       </c>
       <c r="C15" t="n">
-        <v>-2.447090783119101</v>
+        <v>-22.77114703949607</v>
       </c>
       <c r="D15" t="n">
-        <v>2.591343404656541</v>
+        <v>-36.61337421158958</v>
       </c>
       <c r="E15" t="s">
         <v>17</v>
@@ -896,10 +896,10 @@
         <v>14</v>
       </c>
       <c r="C16" t="n">
-        <v>-39.91611073298978</v>
+        <v>24.3224863606699</v>
       </c>
       <c r="D16" t="n">
-        <v>-89.59025782321442</v>
+        <v>-29.11475831121508</v>
       </c>
       <c r="E16" t="s">
         <v>17</v>
@@ -916,10 +916,10 @@
         <v>15</v>
       </c>
       <c r="C17" t="n">
-        <v>-13.6059741872424</v>
+        <v>-5.402572267828766</v>
       </c>
       <c r="D17" t="n">
-        <v>87.43968560451231</v>
+        <v>91.32934791741965</v>
       </c>
       <c r="E17" t="s">
         <v>17</v>
@@ -936,10 +936,10 @@
         <v>16</v>
       </c>
       <c r="C18" t="n">
-        <v>-9.10312145162537</v>
+        <v>-40.67115771967745</v>
       </c>
       <c r="D18" t="n">
-        <v>13.59593024948138</v>
+        <v>-87.53396823192645</v>
       </c>
       <c r="E18" t="s">
         <v>17</v>
@@ -956,10 +956,10 @@
         <v>17</v>
       </c>
       <c r="C19" t="n">
-        <v>26.17179564370285</v>
+        <v>-0.4368505723745884</v>
       </c>
       <c r="D19" t="n">
-        <v>-35.76449135823198</v>
+        <v>9.432466320620222</v>
       </c>
       <c r="E19" t="s">
         <v>17</v>
@@ -976,10 +976,10 @@
         <v>18</v>
       </c>
       <c r="C20" t="n">
-        <v>3.548724135704674</v>
+        <v>-16.72196598646099</v>
       </c>
       <c r="D20" t="n">
-        <v>-37.01012112572288</v>
+        <v>43.45888310351546</v>
       </c>
       <c r="E20" t="s">
         <v>17</v>
@@ -996,10 +996,10 @@
         <v>19</v>
       </c>
       <c r="C21" t="n">
-        <v>-45.72639341354221</v>
+        <v>15.29634713476852</v>
       </c>
       <c r="D21" t="n">
-        <v>-64.60699725731783</v>
+        <v>-83.04313422864848</v>
       </c>
       <c r="E21" t="s">
         <v>17</v>
@@ -1016,10 +1016,10 @@
         <v>20</v>
       </c>
       <c r="C22" t="n">
-        <v>15.47473036233153</v>
+        <v>37.01032927000048</v>
       </c>
       <c r="D22" t="n">
-        <v>-19.07164464498223</v>
+        <v>14.28531620098244</v>
       </c>
       <c r="E22" t="s">
         <v>17</v>
@@ -1036,10 +1036,10 @@
         <v>21</v>
       </c>
       <c r="C23" t="n">
-        <v>42.19946580172682</v>
+        <v>5.831376134756006</v>
       </c>
       <c r="D23" t="n">
-        <v>74.16432818162795</v>
+        <v>-14.57852141958386</v>
       </c>
       <c r="E23" t="s">
         <v>17</v>
@@ -1056,10 +1056,10 @@
         <v>22</v>
       </c>
       <c r="C24" t="n">
-        <v>11.36092669010599</v>
+        <v>41.12394811855083</v>
       </c>
       <c r="D24" t="n">
-        <v>-76.26939573709377</v>
+        <v>60.41378758903392</v>
       </c>
       <c r="E24" t="s">
         <v>17</v>
@@ -1076,10 +1076,10 @@
         <v>23</v>
       </c>
       <c r="C25" t="n">
-        <v>-24.82091293894687</v>
+        <v>-44.89685426926108</v>
       </c>
       <c r="D25" t="n">
-        <v>49.83916472955462</v>
+        <v>72.48911130599336</v>
       </c>
       <c r="E25" t="s">
         <v>17</v>
@@ -1096,10 +1096,10 @@
         <v>24</v>
       </c>
       <c r="C26" t="n">
-        <v>18.37217291828543</v>
+        <v>-34.31380334221465</v>
       </c>
       <c r="D26" t="n">
-        <v>24.80290404671575</v>
+        <v>80.36361379626152</v>
       </c>
       <c r="E26" t="s">
         <v>17</v>
@@ -1141,7 +1141,7 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>104.5829775889917</v>
+        <v>106.5456748982687</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1152,7 +1152,7 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>61.9654847667875</v>
+        <v>73.89752703384607</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1163,7 +1163,7 @@
         <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>71.00834208927171</v>
+        <v>57.92193386035419</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -1174,7 +1174,7 @@
         <v>3</v>
       </c>
       <c r="C5" t="n">
-        <v>102.1323052223888</v>
+        <v>6.802317084858752</v>
       </c>
     </row>
     <row r="6" spans="1:3">
@@ -1185,7 +1185,7 @@
         <v>4</v>
       </c>
       <c r="C6" t="n">
-        <v>85.12384449268366</v>
+        <v>46.31010965981822</v>
       </c>
     </row>
     <row r="7" spans="1:3">
@@ -1196,7 +1196,7 @@
         <v>5</v>
       </c>
       <c r="C7" t="n">
-        <v>77.51395401914888</v>
+        <v>73.10443797153236</v>
       </c>
     </row>
     <row r="8" spans="1:3">
@@ -1207,7 +1207,7 @@
         <v>6</v>
       </c>
       <c r="C8" t="n">
-        <v>28.92244249308711</v>
+        <v>49.38195201450795</v>
       </c>
     </row>
     <row r="9" spans="1:3">
@@ -1218,7 +1218,7 @@
         <v>7</v>
       </c>
       <c r="C9" t="n">
-        <v>57.19828906317157</v>
+        <v>69.98570443035528</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1229,7 +1229,7 @@
         <v>8</v>
       </c>
       <c r="C10" t="n">
-        <v>48.9199220671023</v>
+        <v>98.62043964575052</v>
       </c>
     </row>
     <row r="11" spans="1:3">
@@ -1240,7 +1240,7 @@
         <v>9</v>
       </c>
       <c r="C11" t="n">
-        <v>75.33121099590072</v>
+        <v>27.53711867095363</v>
       </c>
     </row>
     <row r="12" spans="1:3">
@@ -1251,7 +1251,7 @@
         <v>10</v>
       </c>
       <c r="C12" t="n">
-        <v>46.0612601290569</v>
+        <v>76.0357221648465</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -1262,7 +1262,7 @@
         <v>11</v>
       </c>
       <c r="C13" t="n">
-        <v>11.86042758978058</v>
+        <v>29.66757213645581</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1273,7 +1273,7 @@
         <v>12</v>
       </c>
       <c r="C14" t="n">
-        <v>52.77480993080396</v>
+        <v>39.12139459322662</v>
       </c>
     </row>
     <row r="15" spans="1:3">
@@ -1284,7 +1284,7 @@
         <v>13</v>
       </c>
       <c r="C15" t="n">
-        <v>2.712014305147573</v>
+        <v>42.07181497767856</v>
       </c>
     </row>
     <row r="16" spans="1:3">
@@ -1295,7 +1295,7 @@
         <v>14</v>
       </c>
       <c r="C16" t="n">
-        <v>98.71819265777106</v>
+        <v>39.36598465453883</v>
       </c>
     </row>
     <row r="17" spans="1:3">
@@ -1306,7 +1306,7 @@
         <v>15</v>
       </c>
       <c r="C17" t="n">
-        <v>88.29274435448015</v>
+        <v>91.08311917838569</v>
       </c>
     </row>
     <row r="18" spans="1:3">
@@ -1317,7 +1317,7 @@
         <v>16</v>
       </c>
       <c r="C18" t="n">
-        <v>16.65599440954206</v>
+        <v>97.02142426461921</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -1328,7 +1328,7 @@
         <v>17</v>
       </c>
       <c r="C19" t="n">
-        <v>43.63750166270777</v>
+        <v>9.645929068109689</v>
       </c>
     </row>
     <row r="20" spans="1:3">
@@ -1339,7 +1339,7 @@
         <v>18</v>
       </c>
       <c r="C20" t="n">
-        <v>35.46164363756871</v>
+        <v>46.39499843045764</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -1350,7 +1350,7 @@
         <v>19</v>
       </c>
       <c r="C21" t="n">
-        <v>80.89494868450986</v>
+        <v>84.06699852812513</v>
       </c>
     </row>
     <row r="22" spans="1:3">
@@ -1361,7 +1361,7 @@
         <v>20</v>
       </c>
       <c r="C22" t="n">
-        <v>24.2314259715583</v>
+        <v>39.3699828767349</v>
       </c>
     </row>
     <row r="23" spans="1:3">
@@ -1372,7 +1372,7 @@
         <v>21</v>
       </c>
       <c r="C23" t="n">
-        <v>86.68066924689877</v>
+        <v>15.08660231552476</v>
       </c>
     </row>
     <row r="24" spans="1:3">
@@ -1383,7 +1383,7 @@
         <v>22</v>
       </c>
       <c r="C24" t="n">
-        <v>77.78161804821913</v>
+        <v>72.64484137651345</v>
       </c>
     </row>
     <row r="25" spans="1:3">
@@ -1394,7 +1394,7 @@
         <v>23</v>
       </c>
       <c r="C25" t="n">
-        <v>55.52592106354519</v>
+        <v>86.09220555690713</v>
       </c>
     </row>
     <row r="26" spans="1:3">
@@ -1405,7 +1405,7 @@
         <v>24</v>
       </c>
       <c r="C26" t="n">
-        <v>30.88798407885472</v>
+        <v>87.90710633663716</v>
       </c>
     </row>
   </sheetData>

</xml_diff>